<commit_message>
Finalize Phase 1 baseline analysis
</commit_message>
<xml_diff>
--- a/2 Output/Phase1_Baseline_Executive/tables/phase1_baseline_jlos_expanded_analysis.xlsx
+++ b/2 Output/Phase1_Baseline_Executive/tables/phase1_baseline_jlos_expanded_analysis.xlsx
@@ -194,7 +194,7 @@
     <t>Knows/explains pathway</t>
   </si>
   <si>
-    <t>district_scto</t>
+    <t>canonical_district</t>
   </si>
   <si>
     <t>Bushenyi</t>
@@ -365,10 +365,10 @@
         <v>11</v>
       </c>
       <c r="C2" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D2" s="1">
-        <v>95.488721804511272</v>
+        <v>88.372093023255815</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
@@ -382,10 +382,10 @@
         <v>12</v>
       </c>
       <c r="C3" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D3" s="1">
-        <v>82.957392720911742</v>
+        <v>86.907837106737986</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
@@ -399,10 +399,10 @@
         <v>13</v>
       </c>
       <c r="C4" s="1">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="D4" s="1">
-        <v>77.819548872180462</v>
+        <v>75.595238095238088</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
@@ -416,10 +416,10 @@
         <v>14</v>
       </c>
       <c r="C5" s="1">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="D5" s="1">
-        <v>73.269230769230759</v>
+        <v>72.154471544715449</v>
       </c>
       <c r="E5" t="s">
         <v>14</v>
@@ -433,10 +433,10 @@
         <v>15</v>
       </c>
       <c r="C6" s="1">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="D6" s="1">
-        <v>70.610687022900763</v>
+        <v>76.446280991735534</v>
       </c>
       <c r="E6" t="s">
         <v>15</v>
@@ -450,10 +450,10 @@
         <v>16</v>
       </c>
       <c r="C7" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D7" s="1">
-        <v>59.586466165413533</v>
+        <v>60.852713178294572</v>
       </c>
       <c r="E7" t="s">
         <v>16</v>
@@ -467,10 +467,10 @@
         <v>17</v>
       </c>
       <c r="C8" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D8" s="1">
-        <v>59.022556390977442</v>
+        <v>60.465116279069761</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
@@ -484,10 +484,10 @@
         <v>18</v>
       </c>
       <c r="C9" s="1">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D9" s="1">
-        <v>54.13533834586466</v>
+        <v>48.799999999999997</v>
       </c>
       <c r="E9" t="s">
         <v>18</v>
@@ -501,10 +501,10 @@
         <v>19</v>
       </c>
       <c r="C10" s="1">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="D10" s="1">
-        <v>50</v>
+        <v>45.081967213114751</v>
       </c>
       <c r="E10" t="s">
         <v>19</v>
@@ -544,10 +544,10 @@
         <v>24</v>
       </c>
       <c r="C2" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D2" s="1">
-        <v>84.962406015037601</v>
+        <v>87.596899224806208</v>
       </c>
       <c r="E2" t="s">
         <v>24</v>
@@ -561,10 +561,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D3" s="1">
-        <v>69.172932330827067</v>
+        <v>70.542635658914733</v>
       </c>
       <c r="E3" t="s">
         <v>32</v>
@@ -578,10 +578,10 @@
         <v>26</v>
       </c>
       <c r="C4" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D4" s="1">
-        <v>40.601503759398497</v>
+        <v>48.062015503875969</v>
       </c>
       <c r="E4" t="s">
         <v>33</v>
@@ -595,10 +595,10 @@
         <v>27</v>
       </c>
       <c r="C5" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D5" s="1">
-        <v>18.045112781954881</v>
+        <v>21.70542635658915</v>
       </c>
       <c r="E5" t="s">
         <v>34</v>
@@ -612,10 +612,10 @@
         <v>28</v>
       </c>
       <c r="C6" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D6" s="1">
-        <v>7.518796992481203</v>
+        <v>9.3023255813953494</v>
       </c>
       <c r="E6" t="s">
         <v>35</v>
@@ -629,10 +629,10 @@
         <v>29</v>
       </c>
       <c r="C7" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D7" s="1">
-        <v>4.5112781954887211</v>
+        <v>3.8759689922480618</v>
       </c>
       <c r="E7" t="s">
         <v>36</v>
@@ -646,10 +646,10 @@
         <v>30</v>
       </c>
       <c r="C8" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D8" s="1">
-        <v>0.75187969924812026</v>
+        <v>0</v>
       </c>
       <c r="E8" t="s">
         <v>37</v>
@@ -663,10 +663,10 @@
         <v>31</v>
       </c>
       <c r="C9" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D9" s="1">
-        <v>0.75187969924812026</v>
+        <v>0.77519379844961245</v>
       </c>
       <c r="E9" t="s">
         <v>38</v>
@@ -706,10 +706,10 @@
         <v>40</v>
       </c>
       <c r="C2" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D2" s="1">
-        <v>69.172932330827067</v>
+        <v>47.286821705426362</v>
       </c>
       <c r="E2" t="s">
         <v>40</v>
@@ -723,10 +723,10 @@
         <v>41</v>
       </c>
       <c r="C3" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D3" s="1">
-        <v>60.150375939849617</v>
+        <v>42.63565891472868</v>
       </c>
       <c r="E3" t="s">
         <v>51</v>
@@ -740,10 +740,10 @@
         <v>42</v>
       </c>
       <c r="C4" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D4" s="1">
-        <v>30.075187969924809</v>
+        <v>20.155038759689919</v>
       </c>
       <c r="E4" t="s">
         <v>42</v>
@@ -757,10 +757,10 @@
         <v>43</v>
       </c>
       <c r="C5" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D5" s="1">
-        <v>24.060150375939848</v>
+        <v>19.379844961240309</v>
       </c>
       <c r="E5" t="s">
         <v>43</v>
@@ -774,10 +774,10 @@
         <v>44</v>
       </c>
       <c r="C6" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D6" s="1">
-        <v>5.2631578947368416</v>
+        <v>4.6511627906976747</v>
       </c>
       <c r="E6" t="s">
         <v>44</v>
@@ -791,10 +791,10 @@
         <v>45</v>
       </c>
       <c r="C7" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D7" s="1">
-        <v>3.007518796992481</v>
+        <v>2.3255813953488369</v>
       </c>
       <c r="E7" t="s">
         <v>45</v>
@@ -808,10 +808,10 @@
         <v>46</v>
       </c>
       <c r="C8" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D8" s="1">
-        <v>2.255639097744361</v>
+        <v>4.6511627906976747</v>
       </c>
       <c r="E8" t="s">
         <v>46</v>
@@ -825,10 +825,10 @@
         <v>47</v>
       </c>
       <c r="C9" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D9" s="1">
-        <v>1.503759398496241</v>
+        <v>2.3255813953488369</v>
       </c>
       <c r="E9" t="s">
         <v>47</v>
@@ -842,10 +842,10 @@
         <v>48</v>
       </c>
       <c r="C10" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D10" s="1">
-        <v>0.75187969924812026</v>
+        <v>0.77519379844961245</v>
       </c>
       <c r="E10" t="s">
         <v>48</v>
@@ -859,10 +859,10 @@
         <v>49</v>
       </c>
       <c r="C11" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D11" s="1">
-        <v>0.75187969924812026</v>
+        <v>1.5503875968992249</v>
       </c>
       <c r="E11" t="s">
         <v>49</v>
@@ -876,10 +876,10 @@
         <v>50</v>
       </c>
       <c r="C12" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D12" s="1">
-        <v>15.03759398496241</v>
+        <v>34.108527131782942</v>
       </c>
       <c r="E12" t="s">
         <v>50</v>
@@ -919,10 +919,10 @@
         <v>11</v>
       </c>
       <c r="C2" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D2" s="1">
-        <v>95.488721804511272</v>
+        <v>88.372093023255815</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
@@ -936,10 +936,10 @@
         <v>12</v>
       </c>
       <c r="C3" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D3" s="1">
-        <v>82.957392720911742</v>
+        <v>86.907837106737986</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
@@ -953,10 +953,10 @@
         <v>53</v>
       </c>
       <c r="C4" s="1">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="D4" s="1">
-        <v>75.845864661654133</v>
+        <v>74.206349206349216</v>
       </c>
       <c r="E4" t="s">
         <v>53</v>
@@ -970,10 +970,10 @@
         <v>15</v>
       </c>
       <c r="C5" s="1">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="D5" s="1">
-        <v>70.610687022900763</v>
+        <v>76.446280991735534</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
@@ -987,10 +987,10 @@
         <v>54</v>
       </c>
       <c r="C6" s="1">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D6" s="1">
-        <v>59.304511278195491</v>
+        <v>60.65891472868217</v>
       </c>
       <c r="E6" t="s">
         <v>57</v>
@@ -1004,10 +1004,10 @@
         <v>55</v>
       </c>
       <c r="C7" s="1">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="D7" s="1">
-        <v>52.161654135338353</v>
+        <v>47.222222222222221</v>
       </c>
       <c r="E7" t="s">
         <v>55</v>
@@ -1021,10 +1021,10 @@
         <v>56</v>
       </c>
       <c r="C8" s="1">
-        <v>104</v>
+        <v>84</v>
       </c>
       <c r="D8" s="1">
-        <v>70.192307692307694</v>
+        <v>62.797619047619037</v>
       </c>
       <c r="E8" t="s">
         <v>56</v>
@@ -1097,46 +1097,46 @@
         <v>55</v>
       </c>
       <c r="C2" s="1">
-        <v>0.96363633871078491</v>
+        <v>0.87272727489471436</v>
       </c>
       <c r="D2" s="1">
-        <v>0.82020199298858643</v>
+        <v>0.85757577419281006</v>
       </c>
       <c r="E2" s="1">
-        <v>0.74090909090909096</v>
+        <v>0.72272727272727277</v>
       </c>
       <c r="F2" s="1">
-        <v>0.70370370370370372</v>
+        <v>0.67592592592592593</v>
       </c>
       <c r="G2" s="1">
-        <v>0.5636363636363636</v>
+        <v>0.57727272727272727</v>
       </c>
       <c r="H2" s="1">
-        <v>0.52727272727272723</v>
+        <v>0.55454545454545456</v>
       </c>
       <c r="I2" s="1">
-        <v>0.53181818181818186</v>
+        <v>0.49545454545454548</v>
       </c>
       <c r="J2" s="1">
-        <v>0.48584905660377359</v>
+        <v>0.42307692307692307</v>
       </c>
       <c r="K2" s="1">
-        <v>0.70454545454545459</v>
+        <v>0.65714285714285714</v>
       </c>
       <c r="L2" s="1">
-        <v>0.72222222222222221</v>
+        <v>0.67647058823529416</v>
       </c>
       <c r="M2" s="1">
-        <v>0.62838202714920044</v>
+        <v>0.61250001192092896</v>
       </c>
       <c r="N2" s="1">
         <v>2.2909090518951416</v>
       </c>
       <c r="O2" s="1">
-        <v>2.3090908527374268</v>
+        <v>1.6181818246841431</v>
       </c>
       <c r="P2" s="1">
-        <v>0.018181817606091499</v>
+        <v>0.27272728085517883</v>
       </c>
     </row>
     <row r="3">
@@ -1144,49 +1144,49 @@
         <v>60</v>
       </c>
       <c r="B3" s="1">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C3" s="1">
-        <v>0.9523809552192688</v>
+        <v>0.92500001192092896</v>
       </c>
       <c r="D3" s="1">
-        <v>0.85978835821151733</v>
+        <v>0.88472223281860352</v>
       </c>
       <c r="E3" s="1">
-        <v>0.8571428571428571</v>
+        <v>0.82051282051282048</v>
       </c>
       <c r="F3" s="1">
-        <v>0.76785714285714291</v>
+        <v>0.76923076923076927</v>
       </c>
       <c r="G3" s="1">
-        <v>0.65476190476190477</v>
+        <v>0.66874999999999996</v>
       </c>
       <c r="H3" s="1">
-        <v>0.6785714285714286</v>
+        <v>0.67500000000000004</v>
       </c>
       <c r="I3" s="1">
-        <v>0.5357142857142857</v>
+        <v>0.5</v>
       </c>
       <c r="J3" s="1">
-        <v>0.51190476190476186</v>
+        <v>0.48717948717948717</v>
       </c>
       <c r="K3" s="1">
-        <v>0.76923076923076927</v>
+        <v>0.72499999999999998</v>
       </c>
       <c r="L3" s="1">
-        <v>0.69999999999999996</v>
+        <v>0.65217391304347827</v>
       </c>
       <c r="M3" s="1">
-        <v>0.6879960298538208</v>
+        <v>0.66387647390365601</v>
       </c>
       <c r="N3" s="1">
-        <v>2.452380895614624</v>
+        <v>2.6500000953674317</v>
       </c>
       <c r="O3" s="1">
-        <v>1.6666666269302368</v>
+        <v>1.2999999523162842</v>
       </c>
       <c r="P3" s="1">
-        <v>0.3333333432674408</v>
+        <v>0.47499999403953552</v>
       </c>
     </row>
     <row r="4">
@@ -1194,49 +1194,49 @@
         <v>61</v>
       </c>
       <c r="B4" s="1">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C4" s="1">
-        <v>0.94444441795349121</v>
+        <v>0.85294115543365479</v>
       </c>
       <c r="D4" s="1">
-        <v>0.80864197015762329</v>
+        <v>0.86928105354309082</v>
       </c>
       <c r="E4" s="1">
-        <v>0.74305555555555558</v>
+        <v>0.734375</v>
       </c>
       <c r="F4" s="1">
-        <v>0.73529411764705888</v>
+        <v>0.7416666666666667</v>
       </c>
       <c r="G4" s="1">
-        <v>0.57638888888888884</v>
+        <v>0.58823529411764708</v>
       </c>
       <c r="H4" s="1">
-        <v>0.58333333333333337</v>
+        <v>0.6029411764705882</v>
       </c>
       <c r="I4" s="1">
-        <v>0.5625</v>
+        <v>0.45967741935483869</v>
       </c>
       <c r="J4" s="1">
-        <v>0.50714285714285712</v>
+        <v>0.45161290322580644</v>
       </c>
       <c r="K4" s="1">
-        <v>0.73076923076923073</v>
+        <v>0.71052631578947367</v>
       </c>
       <c r="L4" s="1">
-        <v>0.83333333333333337</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="M4" s="1">
-        <v>0.64497077465057373</v>
+        <v>0.61548495292663574</v>
       </c>
       <c r="N4" s="1">
-        <v>2</v>
+        <v>2.3529412746429443</v>
       </c>
       <c r="O4" s="1">
-        <v>1.8055555820465088</v>
+        <v>1.3823529481887817</v>
       </c>
       <c r="P4" s="1">
-        <v>0.1388888955116272</v>
+        <v>0.29411765933036804</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Preserve approved baseline report label corrections
</commit_message>
<xml_diff>
--- a/2 Output/Phase1_Baseline_Executive/tables/phase1_baseline_jlos_expanded_analysis.xlsx
+++ b/2 Output/Phase1_Baseline_Executive/tables/phase1_baseline_jlos_expanded_analysis.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="118" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="118" uniqueCount="75">
   <si>
     <t>Advancing Justice Uganda - Phase 1 baseline expanded JLOS analysis</t>
   </si>
@@ -68,10 +68,10 @@
     <t>Referral regularity</t>
   </si>
   <si>
-    <t>Knows where to refer</t>
-  </si>
-  <si>
-    <t>Can explain referral</t>
+    <t>Confidence knowing where to refer</t>
+  </si>
+  <si>
+    <t>Confidence explaining referral</t>
   </si>
   <si>
     <t>Referral documentation</t>
@@ -182,16 +182,13 @@
     <t>Police/court coordination</t>
   </si>
   <si>
-    <t>Knows/explains referral pathway</t>
+    <t>Referral pathway confidence</t>
   </si>
   <si>
     <t>Documentation and feedback</t>
   </si>
   <si>
     <t>Verified referral record</t>
-  </si>
-  <si>
-    <t>Knows/explains pathway</t>
   </si>
   <si>
     <t>canonical_district</t>
@@ -993,7 +990,7 @@
         <v>60.65891472868217</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7">
@@ -1041,57 +1038,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
         <v>20</v>
       </c>
       <c r="C1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" t="s">
         <v>62</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>63</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>64</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>65</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>66</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>67</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>68</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>69</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>70</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>71</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>72</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>73</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>74</v>
-      </c>
-      <c r="P1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2" s="1">
         <v>55</v>
@@ -1141,7 +1138,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="1">
         <v>40</v>
@@ -1191,7 +1188,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B4" s="1">
         <v>34</v>

</xml_diff>